<commit_message>
Questions page: show the portal's last data update date (MK/AL/EN)
Reads meta.sources.questions.lastPortalUpdate and renders it under the page
subtitle, locale-formatted (was only visible on the methodology page).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations.xlsx
+++ b/translations.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D223"/>
+  <dimension ref="A1:D224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2285,3056 +2285,3078 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>mymp.title</t>
+          <t>questions.lastUpdate</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Активност на пратеник</t>
+          <t>Последно освежување на податоците на порталот:</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Aktiviteti i deputetit</t>
+          <t>Përditësimi i fundit i të dhënave në portal:</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>MP activity</t>
+          <t>Data last updated on the portal:</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>mymp.subtitle</t>
+          <t>mymp.title</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Активност на пратениците за периодот јануари–јуни 2025</t>
+          <t>Активност на пратеник</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Aktiviteti i deputetëve për periudhën janar–qershor 2025</t>
+          <t>Aktiviteti i deputetit</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>MP activity for the period January–June 2025</t>
+          <t>MP activity</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>mymp.stalenessNote</t>
+          <t>mymp.subtitle</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Извештајот е последно освежен во ноември 2025. Податоците се преземени од Порталот за отворени податоци на Собранието на Република Северна Македонија, во формата и содржината во која тие се објавени од Собранието.</t>
+          <t>Активност на пратениците за периодот јануари–јуни 2025</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Raporti është përditësuar për herë të fundit në nëntor 2025. Të dhënat janë marrë nga Portali i të dhënave të hapura të Kuvendit të Republikës së Maqedonisë së Veriut, në formën dhe përmbajtjen në të cilën janë publikuar nga Kuvendi.</t>
+          <t>Aktiviteti i deputetëve për periudhën janar–qershor 2025</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>The report was last updated in November 2025. Data is sourced from the Open Data Portal of the Assembly of the Republic of North Macedonia, in the form and content in which it is published by the Assembly.</t>
+          <t>MP activity for the period January–June 2025</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>mymp.mostActiveTitle</t>
+          <t>mymp.stalenessNote</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Најактивен пратеник</t>
+          <t>Извештајот е последно освежен во ноември 2025. Податоците се преземени од Порталот за отворени податоци на Собранието на Република Северна Македонија, во формата и содржината во која тие се објавени од Собранието.</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Deputeti më aktiv</t>
+          <t>Raporti është përditësuar për herë të fundit në nëntor 2025. Të dhënat janë marrë nga Portali i të dhënave të hapura të Kuvendit të Republikës së Maqedonisë së Veriut, në formën dhe përmbajtjen në të cilën janë publikuar nga Kuvendi.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Most active MP</t>
+          <t>The report was last updated in November 2025. Data is sourced from the Open Data Portal of the Assembly of the Republic of North Macedonia, in the form and content in which it is published by the Assembly.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>mymp.mostActiveNote</t>
+          <t>mymp.mostActiveTitle</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Рангирано по нормализирана активност низ сите категории · јан–јун 2025</t>
+          <t>Најактивен пратеник</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Renditur sipas aktivitetit të normalizuar në të gjitha kategoritë · jan–qer 2025</t>
+          <t>Deputeti më aktiv</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Ranked by normalised activity across all categories · Jan–Jun 2025</t>
+          <t>Most active MP</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>mymp.kpiMPs</t>
+          <t>mymp.mostActiveNote</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Пратеници</t>
+          <t>Рангирано по нормализирана активност низ сите категории · јан–јун 2025</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Deputetë</t>
+          <t>Renditur sipas aktivitetit të normalizuar në të gjitha kategoritë · jan–qer 2025</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>MPs</t>
+          <t>Ranked by normalised activity across all categories · Jan–Jun 2025</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>mymp.newlySeatedNote</t>
+          <t>mymp.kpiMPs</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>стапиле по извештајниот период</t>
+          <t>Пратеници</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>morën mandat pas raportit</t>
+          <t>Deputetë</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>seated after the report period</t>
+          <t>MPs</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>mymp.noPeriodData</t>
+          <t>mymp.newlySeatedNote</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Стапил на должност по последниот извештај за активност</t>
+          <t>стапиле по извештајниот период</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Ka marrë mandatin pas raportit të fundit të aktivitetit</t>
+          <t>morën mandat pas raportit</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Took office after the latest activity report</t>
+          <t>seated after the report period</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>mymp.kpiAvgAttendance</t>
+          <t>mymp.noPeriodData</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Просечно присуство</t>
+          <t>Стапил на должност по последниот извештај за активност</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Prezenca mesatare</t>
+          <t>Ka marrë mandatin pas raportit të fundit të aktivitetit</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Average attendance</t>
+          <t>Took office after the latest activity report</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>mymp.kpiZeroQuestions</t>
+          <t>mymp.kpiAvgAttendance</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Пратеници без прашања</t>
+          <t>Просечно присуство</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Deputetë pa pyetje</t>
+          <t>Prezenca mesatare</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>MPs with no questions</t>
+          <t>Average attendance</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>mymp.chartAttendance</t>
+          <t>mymp.kpiZeroQuestions</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Присуство на пленарни седници</t>
+          <t>Пратеници без прашања</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Prezenca në seanca plenare</t>
+          <t>Deputetë pa pyetje</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Plenary session attendance</t>
+          <t>MPs with no questions</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>mymp.chartDiscussions</t>
+          <t>mymp.chartAttendance</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Дискусии</t>
+          <t>Присуство на пленарни седници</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Diskutime</t>
+          <t>Prezenca në seanca plenare</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Discussions</t>
+          <t>Plenary session attendance</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>mymp.chartQuestions</t>
+          <t>mymp.chartDiscussions</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Поставени прашања</t>
+          <t>Дискусии</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Pyetje të parashtruara</t>
+          <t>Diskutime</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Questions asked</t>
+          <t>Discussions</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>mymp.colMP</t>
+          <t>mymp.chartQuestions</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Пратеник</t>
+          <t>Поставени прашања</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Deputeti</t>
+          <t>Pyetje të parashtruara</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>Questions asked</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>mymp.colAttendance</t>
+          <t>mymp.colMP</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Присуство</t>
+          <t>Пратеник</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Prezenca</t>
+          <t>Deputeti</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Attendance</t>
+          <t>MP</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>mymp.colExcused</t>
+          <t>mymp.colAttendance</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Оправдано отсуство</t>
+          <t>Присуство</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Mungesë e arsyetuar</t>
+          <t>Prezenca</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Excused absence</t>
+          <t>Attendance</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>mymp.colUnexcused</t>
+          <t>mymp.colExcused</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Неоправдано отсуство</t>
+          <t>Оправдано отсуство</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Mungesa e pa arsyetuar</t>
+          <t>Mungesë e arsyetuar</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Unexcused absence</t>
+          <t>Excused absence</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>mymp.colDiscussions</t>
+          <t>mymp.colUnexcused</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Дискусии</t>
+          <t>Неоправдано отсуство</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Diskutime</t>
+          <t>Mungesa e pa arsyetuar</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Discussions</t>
+          <t>Unexcused absence</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>mymp.colLaws</t>
+          <t>mymp.colDiscussions</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Закони</t>
+          <t>Дискусии</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Ligje</t>
+          <t>Diskutime</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Laws</t>
+          <t>Discussions</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>mymp.colAmendments</t>
+          <t>mymp.colLaws</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Амандмани</t>
+          <t>Закони</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Amendamente</t>
+          <t>Ligje</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Amendments</t>
+          <t>Laws</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>mymp.colQuestions</t>
+          <t>mymp.colAmendments</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Прашања</t>
+          <t>Амандмани</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Pyetje</t>
+          <t>Amendamente</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Questions</t>
+          <t>Amendments</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>mymp.colCommittees</t>
+          <t>mymp.colQuestions</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Комисии</t>
+          <t>Прашања</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Komisione</t>
+          <t>Pyetje</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Committees</t>
+          <t>Questions</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>mymp.zeroQuestionsLabel</t>
+          <t>mymp.colCommittees</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Пратеници кои не поставиле ниту едно прашање</t>
+          <t>Комисии</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Deputetë që nuk kanë parashtruar asnjë pyetje</t>
+          <t>Komisione</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>MPs who asked no questions at all</t>
+          <t>Committees</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>mymp.top5Title</t>
+          <t>mymp.zeroQuestionsLabel</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Топ 5 најактивни пратеници</t>
+          <t>Пратеници кои не поставиле ниту едно прашање</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Top 5 deputetët më aktivë</t>
+          <t>Deputetë që nuk kanë parashtruar asnjë pyetje</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Top 5 most active MPs</t>
+          <t>MPs who asked no questions at all</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>mymp.top15Label</t>
+          <t>mymp.top5Title</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Топ 15 —</t>
+          <t>Топ 5 најактивни пратеници</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Top 15 —</t>
+          <t>Top 5 deputetët më aktivë</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Top 15 —</t>
+          <t>Top 5 most active MPs</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>mymp.compositeLabel</t>
+          <t>mymp.top15Label</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Вкупна активност</t>
+          <t>Топ 15 —</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Aktiviteti i përgjithshëm</t>
+          <t>Top 15 —</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Overall activity</t>
+          <t>Top 15 —</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>mymp.onlyZero</t>
+          <t>mymp.compositeLabel</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Само без прашања</t>
+          <t>Вкупна активност</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Vetëm pa pyetje</t>
+          <t>Aktiviteti i përgjithshëm</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Only without questions</t>
+          <t>Overall activity</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>mymp.zeroSentence</t>
+          <t>mymp.onlyZero</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>{count} од {total} пратеници не поставиле ниту едно прашање во периодот јануари–јуни 2025.</t>
+          <t>Само без прашања</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>{count} nga {total} deputetë nuk kanë parashtruar asnjë pyetje në periudhën janar–qershor 2025.</t>
+          <t>Vetëm pa pyetje</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>{count} of {total} MPs asked no questions at all in the period January–June 2025.</t>
+          <t>Only without questions</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>mymp.periodLabel</t>
+          <t>mymp.zeroSentence</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Период</t>
+          <t>{count} од {total} пратеници не поставиле ниту едно прашање во периодот јануари–јуни 2025.</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Periudha</t>
+          <t>{count} nga {total} deputetë nuk kanë parashtruar asnjë pyetje në periudhën janar–qershor 2025.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>{count} of {total} MPs asked no questions at all in the period January–June 2025.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>offices.title</t>
+          <t>mymp.periodLabel</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Канцеларии за контакт со граѓани</t>
+          <t>Период</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Zyrat e kontaktit me qytetarët</t>
+          <t>Periudha</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Citizen contact offices</t>
+          <t>Period</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>offices.subtitle</t>
+          <t>offices.title</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Статистики за граѓански случаи по канцеларии на пратеници · по состојба со 8 јануари 2026</t>
+          <t>Канцеларии за контакт со граѓани</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Statistika të rasteve të qytetarëve sipas zyrave të deputetëve · sipas gjendjes më 8 janar 2026</t>
+          <t>Zyrat e kontaktit me qytetarët</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Statistics on citizen cases by MP contact offices · as of 8 January 2026</t>
+          <t>Citizen contact offices</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>offices.kpiCases</t>
+          <t>offices.subtitle</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Случаи</t>
+          <t>Статистики за граѓански случаи по канцеларии на пратеници · по состојба со 8 јануари 2026</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Raste</t>
+          <t>Statistika të rasteve të qytetarëve sipas zyrave të deputetëve · sipas gjendjes më 8 janar 2026</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Cases</t>
+          <t>Statistics on citizen cases by MP contact offices · as of 8 January 2026</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>offices.kpiMeetings</t>
+          <t>offices.kpiCases</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Средби</t>
+          <t>Случаи</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Takime</t>
+          <t>Raste</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Meetings</t>
+          <t>Cases</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>offices.kpiEvents</t>
+          <t>offices.kpiMeetings</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Настани</t>
+          <t>Средби</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Ngjarje</t>
+          <t>Takime</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Meetings</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>offices.kpiInitiatives</t>
+          <t>offices.kpiEvents</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Иницијативи</t>
+          <t>Настани</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Iniciativa</t>
+          <t>Ngjarje</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Initiatives</t>
+          <t>Events</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>offices.chartByMP</t>
+          <t>offices.kpiInitiatives</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Случаи по пратеник</t>
+          <t>Иницијативи</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Raste sipas deputetit</t>
+          <t>Iniciativa</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Cases by MP</t>
+          <t>Initiatives</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>offices.chartByType</t>
+          <t>offices.chartByMP</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Случаи по тип</t>
+          <t>Случаи по пратеник</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Raste sipas llojit</t>
+          <t>Raste sipas deputetit</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Cases by type</t>
+          <t>Cases by MP</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>offices.chartByParty</t>
+          <t>offices.chartByType</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Случаи по партија</t>
+          <t>Случаи по тип</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Raste sipas partisë</t>
+          <t>Raste sipas llojit</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Cases by party</t>
+          <t>Cases by type</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>offices.chartByGender</t>
+          <t>offices.chartByParty</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Случаи по пол</t>
+          <t>Случаи по партија</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Raste sipas gjinisë</t>
+          <t>Raste sipas partisë</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Cases by gender</t>
+          <t>Cases by party</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>offices.chartByAge</t>
+          <t>offices.chartByGender</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Случаи по возрасна група</t>
+          <t>Случаи по пол</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Raste sipas grupmoshës</t>
+          <t>Raste sipas gjinisë</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Cases by age group</t>
+          <t>Cases by gender</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>offices.chartByEthnicity</t>
+          <t>offices.chartByAge</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Случаи по етничка припадност</t>
+          <t>Случаи по возрасна група</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Raste sipas përkatësisë etnike</t>
+          <t>Raste sipas grupmoshës</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Cases by ethnicity</t>
+          <t>Cases by age group</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>offices.chartOverTime</t>
+          <t>offices.chartByEthnicity</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Случаи по период</t>
+          <t>Случаи по етничка припадност</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Raste sipas periudhës</t>
+          <t>Raste sipas përkatësisë etnike</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Cases over time</t>
+          <t>Cases by ethnicity</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>offices.chartByAgeNote</t>
+          <t>offices.chartOverTime</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Случаи по возрасна група на граѓаните</t>
+          <t>Случаи по период</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Raste sipas grupmoshës së qytetarëve</t>
+          <t>Raste sipas periudhës</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Cases by age group of citizens</t>
+          <t>Cases over time</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>offices.chartByEthnicityNote</t>
+          <t>offices.chartByAgeNote</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Случаи по етничка припадност на граѓаните</t>
+          <t>Случаи по возрасна група на граѓаните</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Raste sipas përkatësisë etnike të qytetarëve</t>
+          <t>Raste sipas grupmoshës së qytetarëve</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Cases by ethnicity of citizens</t>
+          <t>Cases by age group of citizens</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>offices.male</t>
+          <t>offices.chartByEthnicityNote</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Машки</t>
+          <t>Случаи по етничка припадност на граѓаните</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Meshkuj</t>
+          <t>Raste sipas përkatësisë etnike të qytetarëve</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Cases by ethnicity of citizens</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>offices.female</t>
+          <t>offices.male</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Женски</t>
+          <t>Машки</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Femra</t>
+          <t>Meshkuj</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>offices.formerMP</t>
+          <t>offices.female</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>поранешен пратеник</t>
+          <t>Женски</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ish-deputet</t>
+          <t>Femra</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>former MP</t>
+          <t>Female</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>map.title</t>
+          <t>offices.formerMP</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Локации на канцеларии</t>
+          <t>поранешен пратеник</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Vendndodhjet e zyrave</t>
+          <t>ish-deputet</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Office locations</t>
+          <t>former MP</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>map.locatedSuffix</t>
+          <t>map.title</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>лоцирани канцеларии на мапата</t>
+          <t>Локации на канцеларии</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>zyra të lokalizuara në hartë</t>
+          <t>Vendndodhjet e zyrave</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>offices located on the map</t>
+          <t>Office locations</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>map.popupTitle</t>
+          <t>map.locatedSuffix</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Канцеларија</t>
+          <t>лоцирани канцеларии на мапата</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Zyra</t>
+          <t>zyra të lokalizuara në hartë</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>offices located on the map</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>profile.title</t>
+          <t>map.popupTitle</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Профил на пратеник</t>
+          <t>Канцеларија</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Profili i deputetit</t>
+          <t>Zyra</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>MP profile</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>profile.subtitle</t>
+          <t>profile.title</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Прашања 2024–2028 · Активност јануари–јуни 2025 · Канцеларии по состојба со 8 јануари 2026</t>
+          <t>Профил на пратеник</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Pyetje 2024–2028 · Aktiviteti janar–qershor 2025 · Zyrat sipas gjendjes më 8 janar 2026</t>
+          <t>Profili i deputetit</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Questions 2024–2028 · Activity January–June 2025 · Offices as of 8 January 2026</t>
+          <t>MP profile</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>profile.sectionQuestions</t>
+          <t>profile.subtitle</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Парламентарни прашања</t>
+          <t>Прашања 2024–2028 · Активност јануари–јуни 2025 · Канцеларии по состојба со 8 јануари 2026</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Pyetje parlamentare</t>
+          <t>Pyetje 2024–2028 · Aktiviteti janar–qershor 2025 · Zyrat sipas gjendjes më 8 janar 2026</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Parliamentary questions</t>
+          <t>Questions 2024–2028 · Activity January–June 2025 · Offices as of 8 January 2026</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>profile.sectionActivity</t>
+          <t>profile.sectionQuestions</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Активност во Собранието</t>
+          <t>Парламентарни прашања</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Aktiviteti në Kuvend</t>
+          <t>Pyetje parlamentare</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Activity in the Assembly</t>
+          <t>Parliamentary questions</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>profile.sectionOffice</t>
+          <t>profile.sectionActivity</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Канцеларија за контакт</t>
+          <t>Активност во Собранието</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Zyra e kontaktit</t>
+          <t>Aktiviteti në Kuvend</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Contact office</t>
+          <t>Activity in the Assembly</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>profile.noOfficeData</t>
+          <t>profile.sectionOffice</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Овој пратеник нема евидентирани граѓански случаи.</t>
+          <t>Канцеларија за контакт</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Ky deputet nuk ka raste të qytetarëve të evidentuara.</t>
+          <t>Zyra e kontaktit</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>This MP has no recorded citizen cases.</t>
+          <t>Contact office</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>profile.noQuestionsData</t>
+          <t>profile.noOfficeData</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Овој пратеник не поставил прашања во тековниот мандат.</t>
+          <t>Овој пратеник нема евидентирани граѓански случаи.</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Ky deputet nuk ka parashtruar pyetje në mandatin aktual.</t>
+          <t>Ky deputet nuk ka raste të qytetarëve të evidentuara.</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>This MP asked no questions in the current mandate.</t>
+          <t>This MP has no recorded citizen cases.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>profile.questionsAsked</t>
+          <t>profile.noQuestionsData</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Поставени прашања</t>
+          <t>Овој пратеник не поставил прашања во тековниот мандат.</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Pyetje të parashtruara</t>
+          <t>Ky deputet nuk ka parashtruar pyetje në mandatin aktual.</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Questions asked</t>
+          <t>This MP asked no questions in the current mandate.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>profile.plenaryAttendance</t>
+          <t>profile.questionsAsked</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Присуство на пленарни седници</t>
+          <t>Поставени прашања</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Prezenca në seanca plenare</t>
+          <t>Pyetje të parashtruara</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Plenary session attendance</t>
+          <t>Questions asked</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>profile.committees</t>
+          <t>profile.plenaryAttendance</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Комисии</t>
+          <t>Присуство на пленарни седници</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Komisione</t>
+          <t>Prezenca në seanca plenare</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Committees</t>
+          <t>Plenary session attendance</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>profile.citizenCases</t>
+          <t>profile.committees</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Граѓански случаи</t>
+          <t>Комисии</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Raste qytetare</t>
+          <t>Komisione</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Citizen cases</t>
+          <t>Committees</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>profile.topInstitutions</t>
+          <t>profile.citizenCases</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Најчесто адресирани институции</t>
+          <t>Граѓански случаи</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Institucionet më të adresuara</t>
+          <t>Raste qytetare</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Most frequently addressed institutions</t>
+          <t>Citizen cases</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>profile.recentQuestions</t>
+          <t>profile.topInstitutions</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Последни прашања</t>
+          <t>Најчесто адресирани институции</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Pyetjet e fundit</t>
+          <t>Institucionet më të adresuara</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Recent questions</t>
+          <t>Most frequently addressed institutions</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>profile.casesByType</t>
+          <t>profile.recentQuestions</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Случаи по тип</t>
+          <t>Последни прашања</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Raste sipas llojit</t>
+          <t>Pyetjet e fundit</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Cases by type</t>
+          <t>Recent questions</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>profile.independentBody</t>
+          <t>profile.casesByType</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Независно тело</t>
+          <t>Случаи по тип</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Organ i pavarur</t>
+          <t>Raste sipas llojit</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Independent body</t>
+          <t>Cases by type</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>profile.sort.name</t>
+          <t>profile.independentBody</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Абецеден ред</t>
+          <t>Независно тело</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Rend alfabetik</t>
+          <t>Organ i pavarur</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Alphabetical</t>
+          <t>Independent body</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>profile.sort.composite</t>
+          <t>profile.sort.name</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Општа активност</t>
+          <t>Абецеден ред</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Aktiviteti i përgjithshëm</t>
+          <t>Rend alfabetik</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Overall activity</t>
+          <t>Alphabetical</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>profile.sort.questions</t>
+          <t>profile.sort.composite</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Прашања (2024–28)</t>
+          <t>Општа активност</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Pyetje (2024–28)</t>
+          <t>Aktiviteti i përgjithshëm</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Questions (2024–28)</t>
+          <t>Overall activity</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>profile.sort.attendance</t>
+          <t>profile.sort.questions</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Присуство</t>
+          <t>Прашања (2024–28)</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Prezenca</t>
+          <t>Pyetje (2024–28)</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Attendance</t>
+          <t>Questions (2024–28)</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>profile.sort.discussions</t>
+          <t>profile.sort.attendance</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Дискусии</t>
+          <t>Присуство</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Diskutime</t>
+          <t>Prezenca</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Discussions</t>
+          <t>Attendance</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>profile.sort.laws</t>
+          <t>profile.sort.discussions</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Закони</t>
+          <t>Дискусии</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Ligje</t>
+          <t>Diskutime</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Laws</t>
+          <t>Discussions</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>profile.sort.amendments</t>
+          <t>profile.sort.laws</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Амандмани</t>
+          <t>Закони</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Amendamente</t>
+          <t>Ligje</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Amendments</t>
+          <t>Laws</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>profile.sort.committees</t>
+          <t>profile.sort.amendments</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Комисии</t>
+          <t>Амандмани</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Komisione</t>
+          <t>Amendamente</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Committees</t>
+          <t>Amendments</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>home.pageTitle</t>
+          <t>profile.sort.committees</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Парламентарни отворени податоци</t>
+          <t>Комисии</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Të dhëna të hapura parlamentare</t>
+          <t>Komisione</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Parliamentary open data</t>
+          <t>Committees</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>home.badge</t>
+          <t>home.pageTitle</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Собрание на Република Северна Македонија · 2024–2028</t>
+          <t>Парламентарни отворени податоци</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Kuvendi i Republikës së Maqedonisë së Veriut · 2024–2028</t>
+          <t>Të dhëna të hapura parlamentare</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Assembly of the Republic of North Macedonia · 2024–2028</t>
+          <t>Parliamentary open data</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>home.heroTitle</t>
+          <t>home.badge</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Интерактивен панел на отворени податоци</t>
+          <t>Собрание на Република Северна Македонија · 2024–2028</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Panel interaktiv i të dhënave të hapura</t>
+          <t>Kuvendi i Republikës së Maqedonisë së Veriut · 2024–2028</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Interactive open data dashboard</t>
+          <t>Assembly of the Republic of North Macedonia · 2024–2028</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>home.heroSubtitle</t>
+          <t>home.heroTitle</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>на Собранието на Република Северна Македонија</t>
+          <t>Интерактивен панел на отворени податоци</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>i Kuvendit të Republikës së Maqedonisë së Veriut</t>
+          <t>Panel interaktiv i të dhënave të hapura</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>of the Assembly of the Republic of North Macedonia</t>
+          <t>Interactive open data dashboard</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>home.kpiQuestions</t>
+          <t>home.heroSubtitle</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Пратенички прашања</t>
+          <t>на Собранието на Република Северна Македонија</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Pyetje deputetësh</t>
+          <t>i Kuvendit të Republikës së Maqedonisë së Veriut</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Parliamentary questions</t>
+          <t>of the Assembly of the Republic of North Macedonia</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>home.kpiQuestionsNote</t>
+          <t>home.kpiQuestions</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>одговорени</t>
+          <t>Пратенички прашања</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>të përgjigjura</t>
+          <t>Pyetje deputetësh</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>answered</t>
+          <t>Parliamentary questions</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>home.kpiMPs</t>
+          <t>home.kpiQuestionsNote</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Пратеници</t>
+          <t>одговорени</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Deputetë</t>
+          <t>të përgjigjura</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>MPs</t>
+          <t>answered</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>home.kpiMPsNote</t>
+          <t>home.kpiMPs</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Активен состав 2024–2028</t>
+          <t>Пратеници</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Përbërja aktive 2024–2028</t>
+          <t>Deputetë</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Active assembly 2024–2028</t>
+          <t>MPs</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>home.kpiOffices</t>
+          <t>home.kpiMPsNote</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Канцеларии</t>
+          <t>Активен состав 2024–2028</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Zyra</t>
+          <t>Përbërja aktive 2024–2028</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Offices</t>
+          <t>Active assembly 2024–2028</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>home.kpiOfficesNote</t>
+          <t>home.kpiOffices</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>за контакт со граѓани</t>
+          <t>Канцеларии</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>për kontakt me qytetarët</t>
+          <t>Zyra</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>for citizen contact</t>
+          <t>Offices</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>home.descQuestions</t>
+          <t>home.kpiOfficesNote</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Прашања поставени до институции, министерства и независни тела во Собранието 2024–2028</t>
+          <t>за контакт со граѓани</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Pyetje të parashtruara institucioneve, ministrive dhe organeve të pavarura në Kuvendin 2024–2028</t>
+          <t>për kontakt me qytetarët</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Questions addressed to institutions, ministries and independent bodies in the Assembly 2024–2028</t>
+          <t>for citizen contact</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>home.descMyMP</t>
+          <t>home.descQuestions</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Присуство, дискусии, закони и амандмани — активност на секој пратеник</t>
+          <t>Прашања поставени до институции, министерства и независни тела во Собранието 2024–2028</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Prezenca, diskutime, ligje dhe amendamente — aktiviteti i secilit deputet</t>
+          <t>Pyetje të parashtruara institucioneve, ministrive dhe organeve të pavarura në Kuvendin 2024–2028</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Attendance, discussions, laws and amendments — the activity of each MP</t>
+          <t>Questions addressed to institutions, ministries and independent bodies in the Assembly 2024–2028</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>home.descOffices</t>
+          <t>home.descMyMP</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Граѓански случаи, состаноци и иницијативи по канцеларии на пратеници</t>
+          <t>Присуство, дискусии, закони и амандмани — активност на секој пратеник</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Raste qytetare, takime dhe iniciativa sipas zyrave të deputetëve</t>
+          <t>Prezenca, diskutime, ligje dhe amendamente — aktiviteti i secilit deputet</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Citizen cases, meetings and initiatives by MP contact offices</t>
+          <t>Attendance, discussions, laws and amendments — the activity of each MP</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>home.descProfile</t>
+          <t>home.descOffices</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Обединет профил на пратеник: парламентарна активност и граѓански случаи</t>
+          <t>Граѓански случаи, состаноци и иницијативи по канцеларии на пратеници</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Profil i unifikuar i deputetit: aktiviteti parlamentar dhe rastet e qytetarëve</t>
+          <t>Raste qytetare, takime dhe iniciativa sipas zyrave të deputetëve</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Unified MP profile: parliamentary activity and citizen cases</t>
+          <t>Citizen cases, meetings and initiatives by MP contact offices</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>home.open</t>
+          <t>home.descProfile</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Отвори</t>
+          <t>Обединет профил на пратеник: парламентарна активност и граѓански случаи</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Hap</t>
+          <t>Profil i unifikuar i deputetit: aktiviteti parlamentar dhe rastet e qytetarëve</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Unified MP profile: parliamentary activity and citizen cases</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>home.disclaimerSupport</t>
+          <t>home.open</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Оваа активност е поддржана од Иницијативата за дигитална демократија на CIVICUS (CIVICUS Digital Democracy Initiative – DDI), а ја спроведува Институтот за демократија „Социетас Цивилис“ – Скопје.</t>
+          <t>Отвори</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Kjo veprimtari mbështetet nga Iniciativa për Demokraci Dixhitale e CIVICUS (CIVICUS Digital Democracy Initiative – DDI), dhe zbatohet nga Instituti për Demokraci „Societas Civilis“ – Shkup.</t>
+          <t>Hap</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>This activity is supported by the CIVICUS Digital Democracy Initiative (DDI) and is implemented by the Institute for Democracy “Societas Civilis” – Skopje.</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>home.disclaimerDataPre</t>
+          <t>home.disclaimerSupport</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Контролната табла користи податоци преземени од</t>
+          <t>Оваа активност е поддржана од Иницијативата за дигитална демократија на CIVICUS (CIVICUS Digital Democracy Initiative – DDI), а ја спроведува Институтот за демократија „Социетас Цивилис“ – Скопје.</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Paneli përdor të dhëna të marra nga</t>
+          <t>Kjo veprimtari mbështetet nga Iniciativa për Demokraci Dixhitale e CIVICUS (CIVICUS Digital Democracy Initiative – DDI), dhe zbatohet nga Instituti për Demokraci „Societas Civilis“ – Shkup.</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>The dashboard uses data sourced from</t>
+          <t>This activity is supported by the CIVICUS Digital Democracy Initiative (DDI) and is implemented by the Institute for Democracy “Societas Civilis” – Skopje.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>home.disclaimerDataPost</t>
+          <t>home.disclaimerDataPre</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>, во формата и содржината во која тие се објавени од Собранието. Институтот за демократија ги презентира и визуелизира достапните податоци, без дополнителна измена или верификација на нивната содржина.</t>
+          <t>Контролната табла користи податоци преземени од</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>, në formën dhe përmbajtjen në të cilën janë publikuar nga Kuvendi. Instituti për Demokraci i prezanton dhe vizualizon të dhënat e disponueshme, pa ndryshim apo verifikim shtesë të përmbajtjes së tyre.</t>
+          <t>Paneli përdor të dhëna të marra nga</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>, in the form and content in which it is published by the Assembly. The Institute for Democracy presents and visualises the available data, without further modification or verification of its content.</t>
+          <t>The dashboard uses data sourced from</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>about.p1</t>
+          <t>home.disclaimerDataPost</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>На својот пат, ИДСЦС има визија за Македонија како високо развиена демократија на слободни и активни граѓани.</t>
+          <t>, во формата и содржината во која тие се објавени од Собранието. Институтот за демократија ги презентира и визуелизира достапните податоци, без дополнителна измена или верификација на нивната содржина.</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Në rrugëtimin e vet, IDSCS ka vizionin për Maqedoninë si një demokraci shumë të zhvilluar të qytetarëve të lirë dhe aktivë.</t>
+          <t>, në formën dhe përmbajtjen në të cilën janë publikuar nga Kuvendi. Instituti për Demokraci i prezanton dhe vizualizon të dhënat e disponueshme, pa ndryshim apo verifikim shtesë të përmbajtjes së tyre.</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>On its journey, IDSCS envisions Macedonia as a highly developed democracy of free and active citizens.</t>
+          <t>, in the form and content in which it is published by the Assembly. The Institute for Democracy presents and visualises the available data, without further modification or verification of its content.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>about.p2</t>
+          <t>about.p1</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Мисијата на ИДСЦС е поддршка на развојот на демократските процеси преку промоција на креирање на политики базирани на истражување, анализи и консултација со засегнатите страни.</t>
+          <t>На својот пат, ИДСЦС има визија за Македонија како високо развиена демократија на слободни и активни граѓани.</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Misioni i IDSCS është mbështetja e zhvillimit të proceseve demokratike përmes promovimit të krijimit të politikave të bazuara në hulumtim, analiza dhe konsultim me palët e interesuara.</t>
+          <t>Në rrugëtimin e vet, IDSCS ka vizionin për Maqedoninë si një demokraci shumë të zhvilluar të qytetarëve të lirë dhe aktivë.</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>The mission of IDSCS is to support the development of democratic processes through promoting policy-making based on research, analysis and consultation with stakeholders.</t>
+          <t>On its journey, IDSCS envisions Macedonia as a highly developed democracy of free and active citizens.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>about.p3</t>
+          <t>about.p2</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>ИДСЦС го истражува развојот на доброто управување, владеењето на правото и европските интеграции на Македонија. ИДСЦС има мисија да ја помогне граѓанската вклученост во носењето на одлуки и да ја зајакне партиципативната политичка култура. Преку зајакнување на слободарските вредности, ИДСЦС придонесува на соживот помеѓу различностите.</t>
+          <t>Мисијата на ИДСЦС е поддршка на развојот на демократските процеси преку промоција на креирање на политики базирани на истражување, анализи и консултација со засегнатите страни.</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>IDSCS hulumton zhvillimin e qeverisjes së mirë, sundimit të së drejtës dhe integrimit evropian të Maqedonisë. IDSCS ka për mision të ndihmojë përfshirjen qytetare në vendimmarrje dhe të forcojë kulturën politike participative. Përmes forcimit të vlerave liridashëse, IDSCS kontribuon në bashkëjetesën mes diversiteteve.</t>
+          <t>Misioni i IDSCS është mbështetja e zhvillimit të proceseve demokratike përmes promovimit të krijimit të politikave të bazuara në hulumtim, analiza dhe konsultim me palët e interesuara.</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>IDSCS researches the development of good governance, the rule of law and Macedonia's European integration. IDSCS has a mission to support citizen involvement in decision-making and to strengthen participative political culture. By reinforcing the values of freedom, IDSCS contributes to coexistence among diversities.</t>
+          <t>The mission of IDSCS is to support the development of democratic processes through promoting policy-making based on research, analysis and consultation with stakeholders.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>about.goalsIntro</t>
+          <t>about.p3</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Во остварувањето на визијата и мисијата, наши долгорочни цели се:</t>
+          <t>ИДСЦС го истражува развојот на доброто управување, владеењето на правото и европските интеграции на Македонија. ИДСЦС има мисија да ја помогне граѓанската вклученост во носењето на одлуки и да ја зајакне партиципативната политичка култура. Преку зајакнување на слободарските вредности, ИДСЦС придонесува на соживот помеѓу различностите.</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Në realizimin e vizionit dhe misionit, qëllimet tona afatgjata janë:</t>
+          <t>IDSCS hulumton zhvillimin e qeverisjes së mirë, sundimit të së drejtës dhe integrimit evropian të Maqedonisë. IDSCS ka për mision të ndihmojë përfshirjen qytetare në vendimmarrje dhe të forcojë kulturën politike participative. Përmes forcimit të vlerave liridashëse, IDSCS kontribuon në bashkëjetesën mes diversiteteve.</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>In pursuing our vision and mission, our long-term goals are:</t>
+          <t>IDSCS researches the development of good governance, the rule of law and Macedonia's European integration. IDSCS has a mission to support citizen involvement in decision-making and to strengthen participative political culture. By reinforcing the values of freedom, IDSCS contributes to coexistence among diversities.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>about.goals.0</t>
+          <t>about.goalsIntro</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Балансиран социо економски развој</t>
+          <t>Во остварувањето на визијата и мисијата, наши долгорочни цели се:</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Zhvillim i balancuar socio-ekonomik</t>
+          <t>Në realizimin e vizionit dhe misionit, qëllimet tona afatgjata janë:</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Balanced socio-economic development</t>
+          <t>In pursuing our vision and mission, our long-term goals are:</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>about.goals.1</t>
+          <t>about.goals.0</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Активна граѓанска вклученост</t>
+          <t>Балансиран социо економски развој</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Përfshirje aktive qytetare</t>
+          <t>Zhvillim i balancuar socio-ekonomik</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Active civic engagement</t>
+          <t>Balanced socio-economic development</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>about.goals.2</t>
+          <t>about.goals.1</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Партиципативна политичка култура</t>
+          <t>Активна граѓанска вклученост</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Kulturë politike participative</t>
+          <t>Përfshirje aktive qytetare</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Participative political culture</t>
+          <t>Active civic engagement</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>about.goals.3</t>
+          <t>about.goals.2</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Остварување на либерални вредности во општеството</t>
+          <t>Партиципативна политичка култура</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Realizimi i vlerave liberale në shoqëri</t>
+          <t>Kulturë politike participative</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Realising liberal values in society</t>
+          <t>Participative political culture</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>about.goals.4</t>
+          <t>about.goals.3</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Почит кон владеење на правото и доброто владеење</t>
+          <t>Остварување на либерални вредности во општеството</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Respekt ndaj sundimit të së drejtës dhe qeverisjes së mirë</t>
+          <t>Realizimi i vlerave liberale në shoqëri</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Respect for the rule of law and good governance</t>
+          <t>Realising liberal values in society</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>about.goals.5</t>
+          <t>about.goals.4</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Промоција на одржливо образование</t>
+          <t>Почит кон владеење на правото и доброто владеење</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Promovimi i arsimit të qëndrueshëm</t>
+          <t>Respekt ndaj sundimit të së drejtës dhe qeverisjes së mirë</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Promotion of sustainable education</t>
+          <t>Respect for the rule of law and good governance</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>about.goals.6</t>
+          <t>about.goals.5</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Остварување на процес на донесување на одлуки заснован на докази</t>
+          <t>Промоција на одржливо образование</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Realizimi i një procesi të vendimmarrjes së bazuar në dëshmi</t>
+          <t>Promovimi i arsimit të qëndrueshëm</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Achieving an evidence-based decision-making process</t>
+          <t>Promotion of sustainable education</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>about.goals.7</t>
+          <t>about.goals.6</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Мултиетничко и мултикултурно сопостоење</t>
+          <t>Остварување на процес на донесување на одлуки заснован на докази</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Bashkëjetesë multietnike dhe multikulturore</t>
+          <t>Realizimi i një procesi të vendimmarrjes së bazuar në dëshmi</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Multi-ethnic and multicultural coexistence</t>
+          <t>Achieving an evidence-based decision-making process</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>project.p1</t>
+          <t>about.goals.7</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Отворените податоци се важна алатка за транспарентност, отчетност и граѓанско учество. Иако Собранието располага со портал за отворени податоци, дел од податоците се објавени во технички формати кои се тешки за користење од пошироката јавност. Ова го ограничува нивниот потенцијал за информирање, анализа и јавен надзор.</t>
+          <t>Мултиетничко и мултикултурно сопостоење</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Të dhënat e hapura janë një mjet i rëndësishëm për transparencë, llogaridhënie dhe pjesëmarrje qytetare. Edhe pse Kuvendi disponon një portal të të dhënave të hapura, një pjesë e të dhënave publikohen në formate teknike që janë të vështira për t'u përdorur nga publiku i gjerë. Kjo kufizon potencialin e tyre për informim, analizë dhe mbikëqyrje publike.</t>
+          <t>Bashkëjetesë multietnike dhe multikulturore</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Open data is an important tool for transparency, accountability and citizen participation. Although the Assembly has an open data portal, some of the data is published in technical formats that are difficult for the general public to use. This limits its potential for information, analysis and public oversight.</t>
+          <t>Multi-ethnic and multicultural coexistence</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>project.p2</t>
+          <t>project.p1</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Проектот „Отворени податоци на Собранието во пракса: Поттикнување граѓанско учество“ има за цел да ги приближи собраниските отворени податоци до граѓаните, медиумите, граѓанските организации, студентите и младите. Проектот комбинира развој на кориснички ориентиран dashboard, практична обука за користење на отворени податоци, дигитална кампања и застапување за одржливост на решението.</t>
+          <t>Отворените податоци се важна алатка за транспарентност, отчетност и граѓанско учество. Иако Собранието располага со портал за отворени податоци, дел од податоците се објавени во технички формати кои се тешки за користење од пошироката јавност. Ова го ограничува нивниот потенцијал за информирање, анализа и јавен надзор.</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Projekti „Të dhënat e hapura të Kuvendit në praktikë: Nxitja e pjesëmarrjes qytetare“ synon t'i afrojë të dhënat e hapura të Kuvendit te qytetarët, mediat, organizatat qytetare, studentët dhe të rinjtë. Projekti kombinon zhvillimin e një paneli të orientuar nga përdoruesi, trajnim praktik për përdorimin e të dhënave të hapura, fushatë dixhitale dhe avokim për qëndrueshmërinë e zgjidhjes.</t>
+          <t>Të dhënat e hapura janë një mjet i rëndësishëm për transparencë, llogaridhënie dhe pjesëmarrje qytetare. Edhe pse Kuvendi disponon një portal të të dhënave të hapura, një pjesë e të dhënave publikohen në formate teknike që janë të vështira për t'u përdorur nga publiku i gjerë. Kjo kufizon potencialin e tyre për informim, analizë dhe mbikëqyrje publike.</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>The project “Assembly Open Data in Practice: Encouraging Citizen Participation” aims to bring the Assembly's open data closer to citizens, the media, civil society organisations, students and young people. The project combines the development of a user-oriented dashboard, practical training in using open data, a digital campaign and advocacy for the sustainability of the solution.</t>
+          <t>Open data is an important tool for transparency, accountability and citizen participation. Although the Assembly has an open data portal, some of the data is published in technical formats that are difficult for the general public to use. This limits its potential for information, analysis and public oversight.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>project.p3</t>
+          <t>project.p2</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Преку проектот ќе се визуелизираат и систематизираат избрани податоци поврзани со пратенички прашања, платформата „Мој пратеник“ и канцелариите за контакт со граѓаните. Истовремено, проектот ќе ги зајакне капацитетите на корисниците за пристапување, толкување и користење на отворени податоци за следење на работата на Собранието и поттикнување поголема јавна отчетност.</t>
+          <t>Проектот „Отворени податоци на Собранието во пракса: Поттикнување граѓанско учество“ има за цел да ги приближи собраниските отворени податоци до граѓаните, медиумите, граѓанските организации, студентите и младите. Проектот комбинира развој на кориснички ориентиран dashboard, практична обука за користење на отворени податоци, дигитална кампања и застапување за одржливост на решението.</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Përmes projektit do të vizualizohen dhe sistematizohen të dhëna të zgjedhura të lidhura me pyetjet e deputetëve, platformën „Deputeti im“ dhe zyrat e kontaktit me qytetarët. Njëkohësisht, projekti do të forcojë kapacitetet e përdoruesve për qasjen, interpretimin dhe përdorimin e të dhënave të hapura për ndjekjen e punës së Kuvendit dhe nxitjen e një llogaridhënieje më të madhe publike.</t>
+          <t>Projekti „Të dhënat e hapura të Kuvendit në praktikë: Nxitja e pjesëmarrjes qytetare“ synon t'i afrojë të dhënat e hapura të Kuvendit te qytetarët, mediat, organizatat qytetare, studentët dhe të rinjtë. Projekti kombinon zhvillimin e një paneli të orientuar nga përdoruesi, trajnim praktik për përdorimin e të dhënave të hapura, fushatë dixhitale dhe avokim për qëndrueshmërinë e zgjidhjes.</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Through the project, selected data related to parliamentary questions, the “My MP” platform and the citizen contact offices will be visualised and systematised. At the same time, the project will strengthen users' capacities to access, interpret and use open data to monitor the work of the Assembly and encourage greater public accountability.</t>
+          <t>The project “Assembly Open Data in Practice: Encouraging Citizen Participation” aims to bring the Assembly's open data closer to citizens, the media, civil society organisations, students and young people. The project combines the development of a user-oriented dashboard, practical training in using open data, a digital campaign and advocacy for the sustainability of the solution.</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>project.p4</t>
+          <t>project.p3</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Отворени податоци на Собранието во пракса: Поттикнување граѓанско учество е поддржан преку грантовата шема Digital Spark, како дел од проектот Regional Support Mechanism EECA, спроведуван од Фондацијата Метаморфозис и TechSoup, во партнерство со CIVICUS и во рамки на Digital Democracy Initiative (DDI), која го опфаќа Глобалниот југ.</t>
+          <t>Преку проектот ќе се визуелизираат и систематизираат избрани податоци поврзани со пратенички прашања, платформата „Мој пратеник“ и канцелариите за контакт со граѓаните. Истовремено, проектот ќе ги зајакне капацитетите на корисниците за пристапување, толкување и користење на отворени податоци за следење на работата на Собранието и поттикнување поголема јавна отчетност.</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Të dhënat e hapura të Kuvendit në praktikë: Nxitja e pjesëmarrjes qytetare mbështetet përmes skemës së granteve Digital Spark, si pjesë e projektit Regional Support Mechanism EECA, i zbatuar nga Fondacioni Metamorphosis dhe TechSoup, në partneritet me CIVICUS dhe në kuadër të Digital Democracy Initiative (DDI), e cila mbulon Jugun Global.</t>
+          <t>Përmes projektit do të vizualizohen dhe sistematizohen të dhëna të zgjedhura të lidhura me pyetjet e deputetëve, platformën „Deputeti im“ dhe zyrat e kontaktit me qytetarët. Njëkohësisht, projekti do të forcojë kapacitetet e përdoruesve për qasjen, interpretimin dhe përdorimin e të dhënave të hapura për ndjekjen e punës së Kuvendit dhe nxitjen e një llogaridhënieje më të madhe publike.</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Assembly Open Data in Practice: Encouraging Citizen Participation, is supported through the Digital Spark granting scheme, as part of the Regional Support Mechanism EECA project, implemented by Metamorphosis Foundation and TechSoup, in partnership with CIVICUS and under the Digital Democracy Initiative (DDI) that covers the Global South.</t>
+          <t>Through the project, selected data related to parliamentary questions, the “My MP” platform and the citizen contact offices will be visualised and systematised. At the same time, the project will strengthen users' capacities to access, interpret and use open data to monitor the work of the Assembly and encourage greater public accountability.</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>methodology.title</t>
+          <t>project.p4</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Методологија</t>
+          <t>Отворени податоци на Собранието во пракса: Поттикнување граѓанско учество е поддржан преку грантовата шема Digital Spark, како дел од проектот Regional Support Mechanism EECA, спроведуван од Фондацијата Метаморфозис и TechSoup, во партнерство со CIVICUS и во рамки на Digital Democracy Initiative (DDI), која го опфаќа Глобалниот југ.</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Metodologjia</t>
+          <t>Të dhënat e hapura të Kuvendit në praktikë: Nxitja e pjesëmarrjes qytetare mbështetet përmes skemës së granteve Digital Spark, si pjesë e projektit Regional Support Mechanism EECA, i zbatuar nga Fondacioni Metamorphosis dhe TechSoup, në partneritet me CIVICUS dhe në kuadër të Digital Democracy Initiative (DDI), e cila mbulon Jugun Global.</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Methodology</t>
+          <t>Assembly Open Data in Practice: Encouraging Citizen Participation, is supported through the Digital Spark granting scheme, as part of the Regional Support Mechanism EECA project, implemented by Metamorphosis Foundation and TechSoup, in partnership with CIVICUS and under the Digital Democracy Initiative (DDI) that covers the Global South.</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>methodology.subtitle</t>
+          <t>methodology.title</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Извори, ограничувања и процес на освежување</t>
+          <t>Методологија</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Burimet, kufizimet dhe procesi i përditësimit</t>
+          <t>Metodologjia</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Sources, limitations and the update process</t>
+          <t>Methodology</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>methodology.formatLabel</t>
+          <t>methodology.subtitle</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Формат</t>
+          <t>Извори, ограничувања и процес на освежување</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Formati</t>
+          <t>Burimet, kufizimet dhe procesi i përditësimit</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Format</t>
+          <t>Sources, limitations and the update process</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>methodology.recordsLabel</t>
+          <t>methodology.formatLabel</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>записи</t>
+          <t>Формат</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>regjistrime</t>
+          <t>Formati</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>records</t>
+          <t>Format</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>methodology.lastPortalUpdate</t>
+          <t>methodology.recordsLabel</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Последно освежување на порталот</t>
+          <t>записи</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Përditësimi i fundit i portalit</t>
+          <t>regjistrime</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Last portal update</t>
+          <t>records</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>methodology.sources.0.name</t>
+          <t>methodology.lastPortalUpdate</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Пратенички прашања 2024–2028</t>
+          <t>Последно освежување на порталот</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Pyetjet e deputetëve 2024–2028</t>
+          <t>Përditësimi i fundit i portalit</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Parliamentary questions 2024–2028</t>
+          <t>Last portal update</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>methodology.sources.0.notes.0</t>
+          <t>methodology.sources.0.name</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Датумите се во .NET legacy формат /Date(ms)/ — конвертирани во ISO-8601.</t>
+          <t>Пратенички прашања 2024–2028</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Datat janë në formatin legacy .NET /Date(ms)/ — të konvertuara në ISO-8601.</t>
+          <t>Pyetjet e deputetëve 2024–2028</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Dates are in the .NET legacy format /Date(ms)/ — converted to ISO-8601.</t>
+          <t>Parliamentary questions 2024–2028</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>methodology.sources.0.notes.1</t>
+          <t>methodology.sources.0.notes.0</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>168 записи (26%) немаат назначена седница — прашањата сè уште не се распоредени.</t>
+          <t>Датумите се во .NET legacy формат /Date(ms)/ — конвертирани во ISO-8601.</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>168 regjistrime (26%) nuk kanë seancë të caktuar — pyetjet ende nuk janë renditur.</t>
+          <t>Datat janë në formatin legacy .NET /Date(ms)/ — të konvertuara në ISO-8601.</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>168 records (26%) have no assigned session — the questions are not yet scheduled.</t>
+          <t>Dates are in the .NET legacy format /Date(ms)/ — converted to ISO-8601.</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>methodology.sources.0.notes.2</t>
+          <t>methodology.sources.0.notes.1</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>91 записи немаат назначена институција — адресирани до независни тела.</t>
+          <t>168 записи (26%) немаат назначена седница — прашањата сè уште не се распоредени.</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>91 regjistrime nuk kanë institucion të caktuar — të adresuara organeve të pavarura.</t>
+          <t>168 regjistrime (26%) nuk kanë seancë të caktuar — pyetjet ende nuk janë renditur.</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>91 records have no assigned institution — addressed to independent bodies.</t>
+          <t>168 records (26%) have no assigned session — the questions are not yet scheduled.</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>methodology.sources.0.notes.3</t>
+          <t>methodology.sources.0.notes.2</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>5 записи со статус 'Одговорено' имаат празен одговор — ограничување на изворните податоци.</t>
+          <t>91 записи немаат назначена институција — адресирани до независни тела.</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>5 regjistrime me status 'Përgjigjur' kanë përgjigje bosh — kufizim i të dhënave burimore.</t>
+          <t>91 regjistrime nuk kanë institucion të caktuar — të adresuara organeve të pavarura.</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>5 records with status 'Answered' have an empty answer — a limitation of the source data.</t>
+          <t>91 records have no assigned institution — addressed to independent bodies.</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>methodology.sources.1.name</t>
+          <t>methodology.sources.0.notes.3</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Мојот пратеник — Извештај бр. 32 (јан–јун 2025)</t>
+          <t>5 записи со статус 'Одговорено' имаат празен одговор — ограничување на изворните податоци.</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Deputeti im — Raporti nr. 32 (jan–qer 2025)</t>
+          <t>5 regjistrime me status 'Përgjigjur' kanë përgjigje bosh — kufizim i të dhënave burimore.</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>My MP — Report no. 32 (Jan–Jun 2025)</t>
+          <t>5 records with status 'Answered' have an empty answer — a limitation of the source data.</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>methodology.sources.1.notes.0</t>
+          <t>methodology.sources.1.name</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Периодичен извештај, не е освежуван од ноември 2025.</t>
+          <t>Мојот пратеник — Извештај бр. 32 (јан–јун 2025)</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Raport periodik, nuk është përditësuar që nga nëntori 2025.</t>
+          <t>Deputeti im — Raporti nr. 32 (jan–qer 2025)</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Periodic report, not updated since November 2025.</t>
+          <t>My MP — Report no. 32 (Jan–Jun 2025)</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>methodology.sources.1.notes.1</t>
+          <t>methodology.sources.1.notes.0</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>XLSX датотеката користи тројна хедер структура со интерни кодови.</t>
+          <t>Периодичен извештај, не е освежуван од ноември 2025.</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Skedari XLSX përdor një strukturë me tre rreshta header me kode të brendshme.</t>
+          <t>Raport periodik, nuk është përditësuar që nga nëntori 2025.</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>The XLSX file uses a three-row header structure with internal codes.</t>
+          <t>Periodic report, not updated since November 2025.</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>methodology.sources.1.notes.2</t>
+          <t>methodology.sources.1.notes.1</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Парсерот ги мапира хедерите по вредност, не по позиција — за отпорност на промени во XLSX структурата.</t>
+          <t>XLSX датотеката користи тројна хедер структура со интерни кодови.</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Parsuesi i mapon header-ët sipas vlerës, jo sipas pozitës — për qëndrueshmëri ndaj ndryshimeve në strukturën XLSX.</t>
+          <t>Skedari XLSX përdor një strukturë me tre rreshta header me kode të brendshme.</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>The parser maps headers by value, not by position — for resilience against changes in the XLSX structure.</t>
+          <t>The XLSX file uses a three-row header structure with internal codes.</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>methodology.sources.2.name</t>
+          <t>methodology.sources.1.notes.2</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Канцеларии за контакт со граѓани</t>
+          <t>Парсерот ги мапира хедерите по вредност, не по позиција — за отпорност на промени во XLSX структурата.</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Zyrat e kontaktit me qytetarët</t>
+          <t>Parsuesi i mapon header-ët sipas vlerës, jo sipas pozitës — për qëndrueshmëri ndaj ndryshimeve në strukturën XLSX.</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Citizen contact offices</t>
+          <t>The parser maps headers by value, not by position — for resilience against changes in the XLSX structure.</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>methodology.sources.2.notes.0</t>
+          <t>methodology.sources.2.name</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Опфаќа 46 пратеници (не сите 120) — само оние со активни канцеларии.</t>
+          <t>Канцеларии за контакт со граѓани</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Përfshin 46 deputetë (jo të gjithë 120) — vetëm ata me zyra aktive.</t>
+          <t>Zyrat e kontaktit me qytetarët</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Covers 46 MPs (not all 120) — only those with active offices.</t>
+          <t>Citizen contact offices</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>methodology.sources.2.notes.1</t>
+          <t>methodology.sources.2.notes.0</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Формат: tidy/long — секоја категорија е засебен ред.</t>
+          <t>Опфаќа 46 пратеници (не сите 120) — само оние со активни канцеларии.</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Format: tidy/long — secila kategori është rresht i veçantë.</t>
+          <t>Përfshin 46 deputetë (jo të gjithë 120) — vetëm ata me zyra aktive.</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Format: tidy/long — each category is a separate row.</t>
+          <t>Covers 46 MPs (not all 120) — only those with active offices.</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>methodology.sources.2.notes.2</t>
+          <t>methodology.sources.2.notes.1</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>UUID идентификаторот се користи за поврзување со другите датасети.</t>
+          <t>Формат: tidy/long — секоја категорија е засебен ред.</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Identifikuesi UUID përdoret për lidhjen me datasetet e tjera.</t>
+          <t>Format: tidy/long — secila kategori është rresht i veçantë.</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>The UUID identifier is used to join with the other datasets.</t>
+          <t>Format: tidy/long — each category is a separate row.</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>methodology.activeAssemblyTitle</t>
+          <t>methodology.sources.2.notes.2</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Активен состав (120 пратеници)</t>
+          <t>UUID идентификаторот се користи за поврзување со другите датасети.</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Përbërja aktive (120 deputetë)</t>
+          <t>Identifikuesi UUID përdoret për lidhjen me datasetet e tjera.</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Active assembly (120 MPs)</t>
+          <t>The UUID identifier is used to join with the other datasets.</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>methodology.activeAssemblyP1</t>
+          <t>methodology.activeAssemblyTitle</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Како единствен извор на вистина за тоа кој е пратеник се користи активниот состав на Собранието — точно 120 членови, преземени од официјалниот регистар на kancelarii.sobranie.mk (статус „активен“). Пратениците кои презедоа функција во Владата или како директори (чиј мандат мирува, пр. премиерот и министрите) и заменетите пратеници не се дел од овие 120 и се исклучени од сите прегледи по пратеник.</t>
+          <t>Активен состав (120 пратеници)</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Si burim i vetëm i së vërtetës për atë se kush është deputet përdoret përbërja aktive e Kuvendit — saktësisht 120 anëtarë, të marrë nga regjistri zyrtar i kancelarii.sobranie.mk (statusi „aktiv“). Deputetët që morën funksion në Qeveri ose si drejtorë (mandati i të cilëve është në qetësi, p.sh. kryeministri dhe ministrat) dhe deputetët e zëvendësuar nuk janë pjesë e këtyre 120 dhe përjashtohen nga të gjitha pamjet sipas deputetit.</t>
+          <t>Përbërja aktive (120 deputetë)</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>The single source of truth for who is an MP is the active assembly of the Assembly — exactly 120 members, sourced from the official register at kancelarii.sobranie.mk (status “active”). MPs who took office in the Government or as directors (whose mandate is frozen, e.g. the prime minister and ministers) and replaced MPs are not part of these 120 and are excluded from all per-MP views.</t>
+          <t>Active assembly (120 MPs)</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>methodology.activeAssemblyP2</t>
+          <t>methodology.activeAssemblyP1</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Извештајот „Мојот пратеник“ се однесува на периодот јануари–јуни 2025; пратениците кои стапиле подоцна (замени) се прикажани во составот, но без податоци за тој период. Записот на пратенички прашања е задржан целосен ({{total}}), но ранг-листите по пратеник ги опфаќаат само активните членови.</t>
+          <t>Како единствен извор на вистина за тоа кој е пратеник се користи активниот состав на Собранието — точно 120 членови, преземени од официјалниот регистар на kancelarii.sobranie.mk (статус „активен“). Пратениците кои презедоа функција во Владата или како директори (чиј мандат мирува, пр. премиерот и министрите) и заменетите пратеници не се дел од овие 120 и се исклучени од сите прегледи по пратеник.</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Raporti „Deputeti im“ i referohet periudhës janar–qershor 2025; deputetët që morën mandatin më vonë (zëvendësime) shfaqen në përbërje, por pa të dhëna për atë periudhë. Regjistri i pyetjeve të deputetëve është mbajtur i plotë ({{total}}), por listat e renditjes sipas deputetit përfshijnë vetëm anëtarët aktivë.</t>
+          <t>Si burim i vetëm i së vërtetës për atë se kush është deputet përdoret përbërja aktive e Kuvendit — saktësisht 120 anëtarë, të marrë nga regjistri zyrtar i kancelarii.sobranie.mk (statusi „aktiv“). Deputetët që morën funksion në Qeveri ose si drejtorë (mandati i të cilëve është në qetësi, p.sh. kryeministri dhe ministrat) dhe deputetët e zëvendësuar nuk janë pjesë e këtyre 120 dhe përjashtohen nga të gjitha pamjet sipas deputetit.</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>The “My MP” report covers the period January–June 2025; MPs who took office later (replacements) are shown in the assembly but without data for that period. The record of parliamentary questions is kept complete ({{total}}), but the per-MP rankings cover only active members.</t>
+          <t>The single source of truth for who is an MP is the active assembly of the Assembly — exactly 120 members, sourced from the official register at kancelarii.sobranie.mk (status “active”). MPs who took office in the Government or as directors (whose mandate is frozen, e.g. the prime minister and ministers) and replaced MPs are not part of these 120 and are excluded from all per-MP views.</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>methodology.joinTitle</t>
+          <t>methodology.activeAssemblyP2</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Поврзување на датасети</t>
+          <t>Извештајот „Мојот пратеник“ се однесува на периодот јануари–јуни 2025; пратениците кои стапиле подоцна (замени) се прикажани во составот, но без податоци за тој период. Записот на пратенички прашања е задржан целосен ({{total}}), но ранг-листите по пратеник ги опфаќаат само активните членови.</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Lidhja e dataseteve</t>
+          <t>Raporti „Deputeti im“ i referohet periudhës janar–qershor 2025; deputetët që morën mandatin më vonë (zëvendësime) shfaqen në përbërje, por pa të dhëna për atë periudhë. Regjistri i pyetjeve të deputetëve është mbajtur i plotë ({{total}}), por listat e renditjes sipas deputetit përfshijnë vetëm anëtarët aktivë.</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Joining the datasets</t>
+          <t>The “My MP” report covers the period January–June 2025; MPs who took office later (replacements) are shown in the assembly but without data for that period. The record of parliamentary questions is kept complete ({{total}}), but the per-MP rankings cover only active members.</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>methodology.joinP1</t>
+          <t>methodology.joinTitle</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Канцелариите содржат UUID идентификатор на пратеник кој се совпаѓа 1:1 со официјалниот регистар и се користи како примарен клуч за поврзување. За другите датасети (имиња во различни формати) се применува детерминистичка нормализација на имиња со експлицитна табела на исклучоци за варијантни записи — без приближно (fuzzy) совпаѓање, за да се избегне погрешно поврзување на различни лица.</t>
+          <t>Поврзување на датасети</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Zyrat përmbajnë një identifikues UUID të deputetit që përputhet 1:1 me regjistrin zyrtar dhe përdoret si çelës primar për lidhjen. Për datasetet e tjera (emra në formate të ndryshme) zbatohet një normalizim deterministik i emrave me një tabelë eksplicite përjashtimesh për regjistrime variantesh — pa përputhje të përafërt (fuzzy), për të shmangur lidhjen e gabuar të personave të ndryshëm.</t>
+          <t>Lidhja e dataseteve</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>The offices contain an MP UUID identifier that matches the official register 1:1 and is used as the primary join key. For the other datasets (names in different formats), a deterministic name normalisation is applied with an explicit exceptions table for variant records — without fuzzy matching, to avoid wrongly joining different people.</t>
+          <t>Joining the datasets</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>methodology.joinP2</t>
+          <t>methodology.joinP1</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Профилот на пратеник ги обединува сите три датасети и покажува каде постојат, а каде недостасуваат податоци.</t>
+          <t>Канцелариите содржат UUID идентификатор на пратеник кој се совпаѓа 1:1 со официјалниот регистар и се користи како примарен клуч за поврзување. За другите датасети (имиња во различни формати) се применува детерминистичка нормализација на имиња со експлицитна табела на исклучоци за варијантни записи — без приближно (fuzzy) совпаѓање, за да се избегне погрешно поврзување на различни лица.</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Profili i deputetit i unifikon të tre datasetet dhe tregon ku ekzistojnë e ku mungojnë të dhënat.</t>
+          <t>Zyrat përmbajnë një identifikues UUID të deputetit që përputhet 1:1 me regjistrin zyrtar dhe përdoret si çelës primar për lidhjen. Për datasetet e tjera (emra në formate të ndryshme) zbatohet një normalizim deterministik i emrave me një tabelë eksplicite përjashtimesh për regjistrime variantesh — pa përputhje të përafërt (fuzzy), për të shmangur lidhjen e gabuar të personave të ndryshëm.</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>The MP profile unifies all three datasets and shows where data exists and where it is missing.</t>
+          <t>The offices contain an MP UUID identifier that matches the official register 1:1 and is used as the primary join key. For the other datasets (names in different formats), a deterministic name normalisation is applied with an explicit exceptions table for variant records — without fuzzy matching, to avoid wrongly joining different people.</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>methodology.refreshTitle</t>
+          <t>methodology.joinP2</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Процес на освежување</t>
+          <t>Профилот на пратеник ги обединува сите три датасети и покажува каде постојат, а каде недостасуваат податоци.</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Procesi i përditësimit</t>
+          <t>Profili i deputetit i unifikon të tre datasetet dhe tregon ku ekzistojnë e ku mungojnë të dhënat.</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Update process</t>
+          <t>The MP profile unifies all three datasets and shows where data exists and where it is missing.</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>methodology.refreshIntro</t>
+          <t>methodology.refreshTitle</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Dashboard-от не користи live feed. Податоците се освежуваат рачно или преку автоматизирана скрипта 2–3 пати до март 2027. При секое освежување:</t>
+          <t>Процес на освежување</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Paneli nuk përdor feed live. Të dhënat përditësohen manualisht ose përmes një skripti të automatizuar 2–3 herë deri në mars 2027. Në çdo përditësim:</t>
+          <t>Procesi i përditësimit</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>The dashboard does not use a live feed. Data is refreshed manually or via an automated script 2–3 times until March 2027. On each refresh:</t>
+          <t>Update process</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>methodology.refreshStep1pre</t>
+          <t>methodology.refreshIntro</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Скриптата</t>
+          <t>Dashboard-от не користи live feed. Податоците се освежуваат рачно или преку автоматизирана скрипта 2–3 пати до март 2027. При секое освежување:</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Skripta</t>
+          <t>Paneli nuk përdor feed live. Të dhënat përditësohen manualisht ose përmes një skripti të automatizuar 2–3 herë deri në mars 2027. Në çdo përditësim:</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>The script</t>
+          <t>The dashboard does not use a live feed. Data is refreshed manually or via an automated script 2–3 times until March 2027. On each refresh:</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>methodology.refreshStep1post</t>
+          <t>methodology.refreshStep1pre</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>ги презема новите датотеки од CKAN API.</t>
+          <t>Скриптата</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>i merr skedarët e rinj nga CKAN API.</t>
+          <t>Skripta</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>fetches the new files from the CKAN API.</t>
+          <t>The script</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>methodology.refreshStep2pre</t>
+          <t>methodology.refreshStep1post</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Скриптата</t>
+          <t>ги презема новите датотеки од CKAN API.</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Skripta</t>
+          <t>i merr skedarët e rinj nga CKAN API.</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>The script</t>
+          <t>fetches the new files from the CKAN API.</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>methodology.refreshStep2post</t>
+          <t>methodology.refreshStep2pre</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>ги обработува и генерира чисти JSON датотеки.</t>
+          <t>Скриптата</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>përpunon dhe gjeneron skedarë JSON të pastër.</t>
+          <t>Skripta</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>processes them and generates clean JSON files.</t>
+          <t>The script</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>methodology.refreshStep3</t>
+          <t>methodology.refreshStep2post</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Системот автоматски го прегради и распоредува dashboard-от.</t>
+          <t>ги обработува и генерира чисти JSON датотеки.</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Sistemi automatikisht e rindërton dhe e publikon panelin.</t>
+          <t>përpunon dhe gjeneron skedarë JSON të pastër.</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>The system automatically rebuilds and deploys the dashboard.</t>
+          <t>processes them and generates clean JSON files.</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
+          <t>methodology.refreshStep3</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Системот автоматски го прегради и распоредува dashboard-от.</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Sistemi automatikisht e rindërton dhe e publikon panelin.</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>The system automatically rebuilds and deploys the dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
           <t>methodology.lastProcessedLabel</t>
         </is>
       </c>
-      <c r="B223" t="inlineStr">
+      <c r="B224" t="inlineStr">
         <is>
           <t>Dashboard последно обработен:</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr">
+      <c r="C224" t="inlineStr">
         <is>
           <t>Paneli i përpunuar së fundi:</t>
         </is>
       </c>
-      <c r="D223" t="inlineStr">
+      <c r="D224" t="inlineStr">
         <is>
           <t>Dashboard last processed:</t>
         </is>

</xml_diff>